<commit_message>
feat(audit): add inspection checks 6, 7, 8 for daily period distribution, Monday P5 off, and Flag/SHL ceremony in CLI and Web tools
</commit_message>
<xml_diff>
--- a/Bao_Cao_Kiem_Dinh_THCS_TKB_FET_V14_DongBo.xlsx
+++ b/Bao_Cao_Kiem_Dinh_THCS_TKB_FET_V14_DongBo.xlsx
@@ -452,28 +452,28 @@
         <v>14</v>
       </c>
       <c r="E2" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F2" t="str">
-        <v>3 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G2" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H2" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I2" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J2" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 3, Thứ 7</v>
       </c>
     </row>
     <row r="3">
@@ -493,16 +493,16 @@
         <v>4 tiết</v>
       </c>
       <c r="F3" t="str">
+        <v>3 tiết</v>
+      </c>
+      <c r="G3" t="str">
+        <v>5 tiết</v>
+      </c>
+      <c r="H3" t="str">
         <v>6 tiết</v>
       </c>
-      <c r="G3" t="str">
-        <v>3 tiết</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2 tiết</v>
-      </c>
       <c r="I3" t="str">
-        <v>5 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J3" t="str">
         <v>NGHỈ</v>
@@ -528,19 +528,19 @@
         <v>19</v>
       </c>
       <c r="E4" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F4" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G4" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H4" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I4" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J4" t="str">
         <v>NGHỈ</v>
@@ -572,10 +572,10 @@
         <v>4 tiết</v>
       </c>
       <c r="G5" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H5" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I5" t="str">
         <v>4 tiết</v>
@@ -607,10 +607,10 @@
         <v>1 tiết</v>
       </c>
       <c r="F6" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G6" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H6" t="str">
         <v>4 tiết</v>
@@ -642,28 +642,28 @@
         <v>18</v>
       </c>
       <c r="E7" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F7" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G7" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H7" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I7" t="str">
         <v>4 tiết</v>
       </c>
       <c r="J7" t="str">
-        <v>NGHỈ</v>
+        <v>4 tiết</v>
       </c>
       <c r="K7">
         <v>1</v>
       </c>
       <c r="L7" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="8">
@@ -689,10 +689,10 @@
         <v>4 tiết</v>
       </c>
       <c r="H8" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I8" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J8" t="str">
         <v>3 tiết</v>
@@ -718,7 +718,7 @@
         <v>16</v>
       </c>
       <c r="E9" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F9" t="str">
         <v>NGHỈ</v>
@@ -730,10 +730,10 @@
         <v>2 tiết</v>
       </c>
       <c r="I9" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J9" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K9">
         <v>1</v>
@@ -759,7 +759,7 @@
         <v>2 tiết</v>
       </c>
       <c r="F10" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G10" t="str">
         <v>4 tiết</v>
@@ -768,7 +768,7 @@
         <v>6 tiết</v>
       </c>
       <c r="I10" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J10" t="str">
         <v>NGHỈ</v>
@@ -803,10 +803,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="H11" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I11" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J11" t="str">
         <v>3 tiết</v>
@@ -835,13 +835,13 @@
         <v>3 tiết</v>
       </c>
       <c r="F12" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G12" t="str">
         <v>2 tiết</v>
       </c>
       <c r="H12" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I12" t="str">
         <v>NGHỈ</v>
@@ -870,22 +870,22 @@
         <v>13</v>
       </c>
       <c r="E13" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F13" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G13" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H13" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I13" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J13" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K13">
         <v>1</v>
@@ -908,7 +908,7 @@
         <v>17</v>
       </c>
       <c r="E14" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F14" t="str">
         <v>3 tiết</v>
@@ -917,7 +917,7 @@
         <v>NGHỈ</v>
       </c>
       <c r="H14" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I14" t="str">
         <v>4 tiết</v>
@@ -946,22 +946,22 @@
         <v>16</v>
       </c>
       <c r="E15" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F15" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G15" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H15" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I15" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J15" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K15">
         <v>1</v>
@@ -984,22 +984,22 @@
         <v>14</v>
       </c>
       <c r="E16" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F16" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="G16" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H16" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I16" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J16" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="K16">
         <v>1</v>
@@ -1022,19 +1022,19 @@
         <v>15</v>
       </c>
       <c r="E17" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F17" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G17" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H17" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I17" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J17" t="str">
         <v>NGHỈ</v>
@@ -1060,22 +1060,22 @@
         <v>15</v>
       </c>
       <c r="E18" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F18" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G18" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H18" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I18" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="J18" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -1098,19 +1098,19 @@
         <v>17</v>
       </c>
       <c r="E19" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F19" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G19" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H19" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I19" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J19" t="str">
         <v>NGHỈ</v>
@@ -1177,7 +1177,7 @@
         <v>3 tiết</v>
       </c>
       <c r="F21" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G21" t="str">
         <v>NGHỈ</v>
@@ -1186,7 +1186,7 @@
         <v>3 tiết</v>
       </c>
       <c r="I21" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J21" t="str">
         <v>4 tiết</v>
@@ -1212,10 +1212,10 @@
         <v>12</v>
       </c>
       <c r="E22" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="F22" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G22" t="str">
         <v>2 tiết</v>
@@ -1230,10 +1230,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 2, Thứ 7</v>
       </c>
     </row>
     <row r="23">
@@ -1250,14 +1250,14 @@
         <v>16</v>
       </c>
       <c r="E23" t="str">
+        <v>1 tiết</v>
+      </c>
+      <c r="F23" t="str">
+        <v>3 tiết</v>
+      </c>
+      <c r="G23" t="str">
         <v>5 tiết</v>
       </c>
-      <c r="F23" t="str">
-        <v>NGHỈ</v>
-      </c>
-      <c r="G23" t="str">
-        <v>4 tiết</v>
-      </c>
       <c r="H23" t="str">
         <v>NGHỈ</v>
       </c>
@@ -1268,10 +1268,10 @@
         <v>3 tiết</v>
       </c>
       <c r="K23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L23" t="str">
-        <v>Thứ 3, Thứ 5</v>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="24">
@@ -1288,28 +1288,28 @@
         <v>14</v>
       </c>
       <c r="E24" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F24" t="str">
-        <v>NGHỈ</v>
+        <v>3 tiết</v>
       </c>
       <c r="G24" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H24" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I24" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J24" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" t="str">
-        <v>Thứ 3</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1326,19 +1326,19 @@
         <v>17</v>
       </c>
       <c r="E25" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F25" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G25" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H25" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I25" t="str">
-        <v>5 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J25" t="str">
         <v>NGHỈ</v>
@@ -1364,19 +1364,19 @@
         <v>17</v>
       </c>
       <c r="E26" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F26" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G26" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H26" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I26" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J26" t="str">
         <v>4 tiết</v>
@@ -1402,19 +1402,19 @@
         <v>15</v>
       </c>
       <c r="E27" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F27" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G27" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H27" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I27" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J27" t="str">
         <v>4 tiết</v>
@@ -1440,16 +1440,16 @@
         <v>16</v>
       </c>
       <c r="E28" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F28" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G28" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H28" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I28" t="str">
         <v>2 tiết</v>
@@ -1478,19 +1478,19 @@
         <v>16</v>
       </c>
       <c r="E29" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F29" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G29" t="str">
         <v>2 tiết</v>
       </c>
       <c r="H29" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I29" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J29" t="str">
         <v>3 tiết</v>
@@ -1516,19 +1516,19 @@
         <v>15</v>
       </c>
       <c r="E30" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F30" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="G30" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H30" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I30" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J30" t="str">
         <v>3 tiết</v>
@@ -1554,28 +1554,28 @@
         <v>11</v>
       </c>
       <c r="E31" t="str">
-        <v>NGHỈ</v>
+        <v>1 tiết</v>
       </c>
       <c r="F31" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G31" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H31" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="I31" t="str">
-        <v>5 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J31" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L31" t="str">
-        <v>Thứ 2, Thứ 5, Thứ 7</v>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="32">
@@ -1592,13 +1592,13 @@
         <v>15</v>
       </c>
       <c r="E32" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F32" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G32" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H32" t="str">
         <v>2 tiết</v>
@@ -1630,19 +1630,19 @@
         <v>20</v>
       </c>
       <c r="E33" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F33" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G33" t="str">
-        <v>3 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="H33" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I33" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J33" t="str">
         <v>NGHỈ</v>
@@ -1709,16 +1709,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F35" t="str">
-        <v>6 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G35" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H35" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I35" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J35" t="str">
         <v>4 tiết</v>
@@ -1744,16 +1744,16 @@
         <v>17</v>
       </c>
       <c r="E36" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F36" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G36" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H36" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I36" t="str">
         <v>NGHỈ</v>
@@ -1788,16 +1788,16 @@
         <v>2 tiết</v>
       </c>
       <c r="G37" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H37" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I37" t="str">
         <v>4 tiết</v>
       </c>
       <c r="J37" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -1861,7 +1861,7 @@
         <v>2 tiết</v>
       </c>
       <c r="F39" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G39" t="str">
         <v>2 tiết</v>
@@ -1873,7 +1873,7 @@
         <v>2 tiết</v>
       </c>
       <c r="J39" t="str">
-        <v>6 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="K39">
         <v>0</v>
@@ -1896,7 +1896,7 @@
         <v>14</v>
       </c>
       <c r="E40" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F40" t="str">
         <v>1 tiết</v>
@@ -1905,7 +1905,7 @@
         <v>2 tiết</v>
       </c>
       <c r="H40" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I40" t="str">
         <v>2 tiết</v>
@@ -1934,28 +1934,28 @@
         <v>16</v>
       </c>
       <c r="E41" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F41" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G41" t="str">
-        <v>NGHỈ</v>
+        <v>1 tiết</v>
       </c>
       <c r="H41" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I41" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J41" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L41" t="str">
-        <v>Thứ 4</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -1975,10 +1975,10 @@
         <v>2 tiết</v>
       </c>
       <c r="F42" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G42" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H42" t="str">
         <v>4 tiết</v>
@@ -2010,28 +2010,28 @@
         <v>21</v>
       </c>
       <c r="E43" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F43" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G43" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H43" t="str">
-        <v>3 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I43" t="str">
-        <v>5 tiết</v>
+        <v>7 tiết</v>
       </c>
       <c r="J43" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" t="str">
-        <v/>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="44">
@@ -2051,25 +2051,25 @@
         <v>3 tiết</v>
       </c>
       <c r="F44" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G44" t="str">
-        <v>2 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="H44" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I44" t="str">
         <v>2 tiết</v>
       </c>
       <c r="J44" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="45">
@@ -2089,16 +2089,16 @@
         <v>4 tiết</v>
       </c>
       <c r="F45" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G45" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H45" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="I45" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J45" t="str">
         <v>4 tiết</v>
@@ -2124,16 +2124,16 @@
         <v>21</v>
       </c>
       <c r="E46" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F46" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G46" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H46" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I46" t="str">
         <v>2 tiết</v>
@@ -2165,13 +2165,13 @@
         <v>3 tiết</v>
       </c>
       <c r="F47" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G47" t="str">
         <v>2 tiết</v>
       </c>
       <c r="H47" t="str">
-        <v>NGHỈ</v>
+        <v>1 tiết</v>
       </c>
       <c r="I47" t="str">
         <v>3 tiết</v>
@@ -2180,10 +2180,10 @@
         <v>3 tiết</v>
       </c>
       <c r="K47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" t="str">
-        <v>Thứ 5</v>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -2200,22 +2200,22 @@
         <v>20</v>
       </c>
       <c r="E48" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F48" t="str">
         <v>5 tiết</v>
       </c>
       <c r="G48" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H48" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I48" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J48" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -2238,28 +2238,28 @@
         <v>17</v>
       </c>
       <c r="E49" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F49" t="str">
         <v>3 tiết</v>
       </c>
       <c r="G49" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H49" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I49" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J49" t="str">
         <v>5 tiết</v>
       </c>
       <c r="K49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" t="str">
-        <v/>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="50">
@@ -2279,7 +2279,7 @@
         <v>3 tiết</v>
       </c>
       <c r="F50" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G50" t="str">
         <v>4 tiết</v>
@@ -2288,16 +2288,16 @@
         <v>NGHỈ</v>
       </c>
       <c r="I50" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J50" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" t="str">
-        <v>Thứ 5</v>
+        <v>Thứ 3, Thứ 5</v>
       </c>
     </row>
     <row r="51">
@@ -2314,22 +2314,22 @@
         <v>16</v>
       </c>
       <c r="E51" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F51" t="str">
-        <v>2 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G51" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H51" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I51" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J51" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="K51">
         <v>1</v>
@@ -2355,7 +2355,7 @@
         <v>2 tiết</v>
       </c>
       <c r="F52" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="G52" t="str">
         <v>4 tiết</v>
@@ -2364,16 +2364,16 @@
         <v>2 tiết</v>
       </c>
       <c r="I52" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J52" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L52" t="str">
-        <v>Thứ 3, Thứ 7</v>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="53">
@@ -2393,19 +2393,19 @@
         <v>2 tiết</v>
       </c>
       <c r="F53" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G53" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H53" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I53" t="str">
         <v>4 tiết</v>
       </c>
       <c r="J53" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="K53">
         <v>0</v>
@@ -2431,10 +2431,10 @@
         <v>3 tiết</v>
       </c>
       <c r="F54" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G54" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H54" t="str">
         <v>2 tiết</v>
@@ -2466,22 +2466,22 @@
         <v>16</v>
       </c>
       <c r="E55" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F55" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G55" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H55" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I55" t="str">
         <v>3 tiết</v>
       </c>
       <c r="J55" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K55">
         <v>0</v>
@@ -2510,10 +2510,10 @@
         <v>2 tiết</v>
       </c>
       <c r="G56" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H56" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I56" t="str">
         <v>2 tiết</v>
@@ -2551,19 +2551,19 @@
         <v>NGHỈ</v>
       </c>
       <c r="H57" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="I57" t="str">
         <v>2 tiết</v>
       </c>
       <c r="J57" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="K57">
         <v>4</v>
       </c>
       <c r="L57" t="str">
-        <v>Thứ 2, Thứ 3, Thứ 4, Thứ 5</v>
+        <v>Thứ 2, Thứ 3, Thứ 4, Thứ 7</v>
       </c>
     </row>
     <row r="58">
@@ -2583,13 +2583,13 @@
         <v>3 tiết</v>
       </c>
       <c r="F58" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G58" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H58" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I58" t="str">
         <v>NGHỈ</v>
@@ -2598,10 +2598,10 @@
         <v>3 tiết</v>
       </c>
       <c r="K58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L58" t="str">
-        <v>Thứ 6</v>
+        <v>Thứ 3, Thứ 6</v>
       </c>
     </row>
     <row r="59">
@@ -2618,28 +2618,28 @@
         <v>15</v>
       </c>
       <c r="E59" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F59" t="str">
         <v>1 tiết</v>
       </c>
       <c r="G59" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H59" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I59" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J59" t="str">
         <v>5 tiết</v>
       </c>
       <c r="K59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="60">
@@ -2656,22 +2656,22 @@
         <v>14</v>
       </c>
       <c r="E60" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F60" t="str">
         <v>1 tiết</v>
       </c>
       <c r="G60" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H60" t="str">
         <v>3 tiết</v>
       </c>
       <c r="I60" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J60" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K60">
         <v>0</v>
@@ -2694,28 +2694,28 @@
         <v>15</v>
       </c>
       <c r="E61" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F61" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G61" t="str">
         <v>1 tiết</v>
       </c>
       <c r="H61" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I61" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J61" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L61" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="62">
@@ -2732,10 +2732,10 @@
         <v>18</v>
       </c>
       <c r="E62" t="str">
-        <v>3 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="F62" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G62" t="str">
         <v>6 tiết</v>
@@ -2744,16 +2744,16 @@
         <v>2 tiết</v>
       </c>
       <c r="I62" t="str">
-        <v>5 tiết</v>
+        <v>7 tiết</v>
       </c>
       <c r="J62" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L62" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 2, Thứ 7</v>
       </c>
     </row>
     <row r="63">
@@ -2773,25 +2773,25 @@
         <v>3 tiết</v>
       </c>
       <c r="F63" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G63" t="str">
         <v>1 tiết</v>
       </c>
       <c r="H63" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I63" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J63" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="K63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="64">
@@ -2817,10 +2817,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="H64" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I64" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J64" t="str">
         <v>3 tiết</v>
@@ -2884,22 +2884,22 @@
         <v>13</v>
       </c>
       <c r="E66" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F66" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G66" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H66" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I66" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J66" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K66">
         <v>0</v>
@@ -2922,22 +2922,22 @@
         <v>16</v>
       </c>
       <c r="E67" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F67" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G67" t="str">
         <v>1 tiết</v>
       </c>
       <c r="H67" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I67" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J67" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K67">
         <v>0</v>
@@ -2998,19 +2998,19 @@
         <v>16</v>
       </c>
       <c r="E69" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F69" t="str">
         <v>4 tiết</v>
       </c>
       <c r="G69" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H69" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I69" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J69" t="str">
         <v>3 tiết</v>
@@ -3074,19 +3074,19 @@
         <v>17</v>
       </c>
       <c r="E71" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F71" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G71" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H71" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I71" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J71" t="str">
         <v>2 tiết</v>
@@ -3112,7 +3112,7 @@
         <v>16</v>
       </c>
       <c r="E72" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F72" t="str">
         <v>4 tiết</v>
@@ -3121,7 +3121,7 @@
         <v>4 tiết</v>
       </c>
       <c r="H72" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I72" t="str">
         <v>2 tiết</v>
@@ -3150,22 +3150,22 @@
         <v>13</v>
       </c>
       <c r="E73" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F73" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="G73" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H73" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I73" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J73" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K73">
         <v>1</v>
@@ -3191,16 +3191,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F74" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G74" t="str">
-        <v>6 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H74" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I74" t="str">
-        <v>4 tiết</v>
+        <v>8 tiết</v>
       </c>
       <c r="J74" t="str">
         <v>NGHỈ</v>
@@ -3226,28 +3226,28 @@
         <v>13</v>
       </c>
       <c r="E75" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F75" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G75" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H75" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I75" t="str">
-        <v>5 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J75" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L75" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 3, Thứ 7</v>
       </c>
     </row>
     <row r="76">
@@ -3264,16 +3264,16 @@
         <v>18</v>
       </c>
       <c r="E76" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F76" t="str">
         <v>3 tiết</v>
       </c>
       <c r="G76" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="H76" t="str">
-        <v>1 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="I76" t="str">
         <v>6 tiết</v>
@@ -3308,10 +3308,10 @@
         <v>2 tiết</v>
       </c>
       <c r="G77" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H77" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I77" t="str">
         <v>2 tiết</v>
@@ -3340,19 +3340,19 @@
         <v>12</v>
       </c>
       <c r="E78" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F78" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G78" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H78" t="str">
         <v>2 tiết</v>
       </c>
       <c r="I78" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J78" t="str">
         <v>NGHỈ</v>
@@ -3378,19 +3378,19 @@
         <v>11</v>
       </c>
       <c r="E79" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F79" t="str">
         <v>1 tiết</v>
       </c>
       <c r="G79" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H79" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I79" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J79" t="str">
         <v>NGHỈ</v>
@@ -3416,7 +3416,7 @@
         <v>19</v>
       </c>
       <c r="E80" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F80" t="str">
         <v>4 tiết</v>
@@ -3428,7 +3428,7 @@
         <v>4 tiết</v>
       </c>
       <c r="I80" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J80" t="str">
         <v>NGHỈ</v>
@@ -3457,16 +3457,16 @@
         <v>3 tiết</v>
       </c>
       <c r="F81" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G81" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H81" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="I81" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J81" t="str">
         <v>3 tiết</v>
@@ -3475,7 +3475,7 @@
         <v>1</v>
       </c>
       <c r="L81" t="str">
-        <v>Thứ 5</v>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="82">
@@ -3492,19 +3492,19 @@
         <v>18</v>
       </c>
       <c r="E82" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F82" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G82" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H82" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I82" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J82" t="str">
         <v>NGHỈ</v>
@@ -3530,7 +3530,7 @@
         <v>14</v>
       </c>
       <c r="E83" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F83" t="str">
         <v>NGHỈ</v>
@@ -3542,7 +3542,7 @@
         <v>2 tiết</v>
       </c>
       <c r="I83" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J83" t="str">
         <v>3 tiết</v>
@@ -3568,22 +3568,22 @@
         <v>17</v>
       </c>
       <c r="E84" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F84" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G84" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H84" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I84" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J84" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K84">
         <v>0</v>
@@ -3606,7 +3606,7 @@
         <v>14</v>
       </c>
       <c r="E85" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F85" t="str">
         <v>2 tiết</v>
@@ -3618,7 +3618,7 @@
         <v>2 tiết</v>
       </c>
       <c r="I85" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J85" t="str">
         <v>3 tiết</v>
@@ -3639,7 +3639,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3675,7 +3675,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Khóa cứng Tiết 5 Thứ 7</v>
+        <v>Khóa cứng Tiết 5 Thứ 7 (Tan sớm)</v>
       </c>
       <c r="B5" t="str">
         <v>ĐẠT 100%</v>
@@ -3691,71 +3691,103 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>Cơ cấu tiết các thứ (T2:4, T3:4, T4:5/4, T5:5, T6:5, T7:4) [Cấu hình]</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>THỐNG KÊ PHÂN BỔ NGÀY NGHỈ</v>
+        <v>Phân bổ số tiết TKB thực tế (K8,9: 27t; K6,7: 26t)</v>
       </c>
       <c r="B8" t="str">
-        <v>SỐ GIÁO VIÊN ĐƯỢC NGHỈ</v>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Thứ 2</v>
+        <v>Nghỉ Tiết 5 Thứ 2 (Tan trường sau Chào cờ chiều)</v>
       </c>
       <c r="B9" t="str">
-        <v>2 giáo viên</v>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Thứ 3</v>
+        <v>Vị trí Chào cờ (T1/T4 T2) &amp; SHL (Tiết 4 T7)</v>
       </c>
       <c r="B10" t="str">
-        <v>13 giáo viên</v>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Thứ 4</v>
+        <v/>
       </c>
       <c r="B11" t="str">
-        <v>14 giáo viên</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Thứ 5</v>
+        <v>THỐNG KÊ PHÂN BỔ NGÀY NGHỈ</v>
       </c>
       <c r="B12" t="str">
-        <v>11 giáo viên</v>
+        <v>SỐ GIÁO VIÊN ĐƯỢC NGHỈ</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Thứ 6</v>
+        <v>Thứ 2</v>
       </c>
       <c r="B13" t="str">
-        <v>8 giáo viên</v>
+        <v>3 giáo viên</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>Thứ 3</v>
+      </c>
+      <c r="B14" t="str">
+        <v>17 giáo viên</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Thứ 4</v>
+      </c>
+      <c r="B15" t="str">
+        <v>14 giáo viên</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Thứ 5</v>
+      </c>
+      <c r="B16" t="str">
+        <v>10 giáo viên</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Thứ 6</v>
+      </c>
+      <c r="B17" t="str">
+        <v>9 giáo viên</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>Thứ 7</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B18" t="str">
         <v>26 giáo viên</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>